<commit_message>
done part tokz dzt
</commit_message>
<xml_diff>
--- a/mode_docx_gen/pmi_tokzdzt/rtponn_modes/РТПО_1.xlsx
+++ b/mode_docx_gen/pmi_tokzdzt/rtponn_modes/РТПО_1.xlsx
@@ -783,39 +783,6 @@
   </sheetPr>
   <dimension ref="A1:AE2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="20" customWidth="1" min="16" max="16"/>
-    <col width="20" customWidth="1" min="17" max="17"/>
-    <col width="20" customWidth="1" min="18" max="18"/>
-    <col width="20" customWidth="1" min="19" max="19"/>
-    <col width="20" customWidth="1" min="20" max="20"/>
-    <col width="20" customWidth="1" min="21" max="21"/>
-    <col width="20" customWidth="1" min="22" max="22"/>
-    <col width="20" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
-    <col width="20" customWidth="1" min="25" max="25"/>
-    <col width="20" customWidth="1" min="26" max="26"/>
-    <col width="20" customWidth="1" min="27" max="27"/>
-    <col width="20" customWidth="1" min="28" max="28"/>
-    <col width="20" customWidth="1" min="29" max="29"/>
-    <col width="20" customWidth="1" min="30" max="30"/>
-    <col width="20" customWidth="1" min="31" max="31"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -865,7 +832,7 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>NaOtkl_hvptoc1_tovctoc</t>
+          <t>NaOtkl_tovctoc</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
@@ -1082,76 +1049,6 @@
   </sheetPr>
   <dimension ref="A1:BP2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="20" customWidth="1" min="16" max="16"/>
-    <col width="20" customWidth="1" min="17" max="17"/>
-    <col width="20" customWidth="1" min="18" max="18"/>
-    <col width="20" customWidth="1" min="19" max="19"/>
-    <col width="20" customWidth="1" min="20" max="20"/>
-    <col width="20" customWidth="1" min="21" max="21"/>
-    <col width="20" customWidth="1" min="22" max="22"/>
-    <col width="20" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
-    <col width="20" customWidth="1" min="25" max="25"/>
-    <col width="20" customWidth="1" min="26" max="26"/>
-    <col width="20" customWidth="1" min="27" max="27"/>
-    <col width="20" customWidth="1" min="28" max="28"/>
-    <col width="20" customWidth="1" min="29" max="29"/>
-    <col width="20" customWidth="1" min="30" max="30"/>
-    <col width="20" customWidth="1" min="31" max="31"/>
-    <col width="20" customWidth="1" min="32" max="32"/>
-    <col width="20" customWidth="1" min="33" max="33"/>
-    <col width="20" customWidth="1" min="34" max="34"/>
-    <col width="20" customWidth="1" min="35" max="35"/>
-    <col width="20" customWidth="1" min="36" max="36"/>
-    <col width="20" customWidth="1" min="37" max="37"/>
-    <col width="20" customWidth="1" min="38" max="38"/>
-    <col width="20" customWidth="1" min="39" max="39"/>
-    <col width="20" customWidth="1" min="40" max="40"/>
-    <col width="20" customWidth="1" min="41" max="41"/>
-    <col width="20" customWidth="1" min="42" max="42"/>
-    <col width="20" customWidth="1" min="43" max="43"/>
-    <col width="20" customWidth="1" min="44" max="44"/>
-    <col width="20" customWidth="1" min="45" max="45"/>
-    <col width="20" customWidth="1" min="46" max="46"/>
-    <col width="20" customWidth="1" min="47" max="47"/>
-    <col width="20" customWidth="1" min="48" max="48"/>
-    <col width="20" customWidth="1" min="49" max="49"/>
-    <col width="20" customWidth="1" min="50" max="50"/>
-    <col width="20" customWidth="1" min="51" max="51"/>
-    <col width="20" customWidth="1" min="52" max="52"/>
-    <col width="20" customWidth="1" min="53" max="53"/>
-    <col width="20" customWidth="1" min="54" max="54"/>
-    <col width="20" customWidth="1" min="55" max="55"/>
-    <col width="20" customWidth="1" min="56" max="56"/>
-    <col width="20" customWidth="1" min="57" max="57"/>
-    <col width="20" customWidth="1" min="58" max="58"/>
-    <col width="20" customWidth="1" min="59" max="59"/>
-    <col width="20" customWidth="1" min="60" max="60"/>
-    <col width="20" customWidth="1" min="61" max="61"/>
-    <col width="20" customWidth="1" min="62" max="62"/>
-    <col width="20" customWidth="1" min="63" max="63"/>
-    <col width="20" customWidth="1" min="64" max="64"/>
-    <col width="20" customWidth="1" min="65" max="65"/>
-    <col width="20" customWidth="1" min="66" max="66"/>
-    <col width="20" customWidth="1" min="67" max="67"/>
-    <col width="20" customWidth="1" min="68" max="68"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -1246,7 +1143,7 @@
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>srab_tovctocc</t>
+          <t>srab_tovctoc</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
@@ -1496,345 +1393,209 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AC2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AD2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AE2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AF2" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AG2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AH2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AI2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AJ2" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AK2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AL2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AM2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AN2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AO2" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AP2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AQ2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AR2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AS2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AT2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AU2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AV2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AW2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AX2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AY2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AZ2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="BA2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="BB2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="BC2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="BD2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="BE2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="BF2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="BG2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="BH2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="BI2" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BJ2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="BK2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="BL2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="BM2" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BN2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="BO2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="BP2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="A2" t="n">
+        <v>0</v>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI2" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM2" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP2" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>